<commit_message>
PBCP rev4: restore per-borehole data, L/NL flags from report FS, BH-03 own SPT data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVMNJXhKJM4HyR9gsSXKh
</commit_message>
<xml_diff>
--- a/deliverables/PBCP-BH-01_rev4.xlsx
+++ b/deliverables/PBCP-BH-01_rev4.xlsx
@@ -12732,8 +12732,10 @@
       <c r="D14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>40</v>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GWL analisis likuefaksi (Report BP-00-GEO-RPT-003)</t>
+        </is>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -12765,13 +12767,15 @@
         <v>45</v>
       </c>
       <c r="C16" s="8">
-        <v>18.5</v>
+        <v>17.8</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>47</v>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report Tabel 5.1</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -12782,13 +12786,15 @@
         <v>49</v>
       </c>
       <c r="C17" s="8">
-        <v>18.399999999999999</v>
+        <v>19.2</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>47</v>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report Tabel 5.1</t>
+        </is>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -12943,8 +12949,10 @@
       <c r="D26" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>70</v>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sesuai perhitungan sebelumnya</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -12958,8 +12966,10 @@
       <c r="D27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>70</v>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sesuai perhitungan sebelumnya</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -13199,7 +13209,11 @@
       <c r="D45" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E45" s="7"/>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DD_max tidak difaktorkan (beban faktor 1,0)</t>
+        </is>
+      </c>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
@@ -13218,12 +13232,16 @@
         <v>9</v>
       </c>
       <c r="C48" s="14">
-        <v>3000</v>
+        <v>5152.9</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E48" s="7"/>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, ASD2(max) - beban lama, update dgn GROUP beban revisi</t>
+        </is>
+      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
@@ -13233,12 +13251,16 @@
         <v>13</v>
       </c>
       <c r="C49" s="14">
-        <v>600</v>
+        <v>1583.9</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E49" s="7"/>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, LRFD3 - beban lama, update dgn GROUP beban revisi</t>
+        </is>
+      </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
@@ -13248,12 +13270,16 @@
         <v>18</v>
       </c>
       <c r="C50" s="14">
-        <v>500</v>
+        <v>1101.5</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E50" s="7"/>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, ASD1 (DL) - beban lama, update dgn GROUP beban revisi</t>
+        </is>
+      </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
@@ -13263,12 +13289,16 @@
         <v>108</v>
       </c>
       <c r="C51" s="14">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E51" s="7"/>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GROUP: tidak ada tiang tarik pada kombinasi yang ditinjau</t>
+        </is>
+      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
@@ -13468,8 +13498,10 @@
       <c r="G7" s="11">
         <v>0</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>128</v>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I7" s="16">
         <f>IF(F7="Clay",Input!$C$32*G7,0)</f>
@@ -13517,8 +13549,10 @@
       <c r="G8" s="11">
         <v>5</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>128</v>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I8" s="20">
         <f>IF(F8="Clay",Input!$C$32*G8,0)</f>
@@ -13568,8 +13602,10 @@
       <c r="G9" s="11">
         <v>18</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>128</v>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I9" s="16">
         <f>IF(F9="Clay",Input!$C$32*G9,0)</f>
@@ -13619,8 +13655,10 @@
       <c r="G10" s="11">
         <v>28</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>128</v>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I10" s="20">
         <f>IF(F10="Clay",Input!$C$32*G10,0)</f>
@@ -13670,8 +13708,10 @@
       <c r="G11" s="11">
         <v>30</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>128</v>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I11" s="16">
         <f>IF(F11="Clay",Input!$C$32*G11,0)</f>
@@ -13721,8 +13761,10 @@
       <c r="G12" s="11">
         <v>35</v>
       </c>
-      <c r="H12" s="22" t="s">
-        <v>128</v>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I12" s="20">
         <f>IF(F12="Clay",Input!$C$32*G12,0)</f>
@@ -13772,8 +13814,10 @@
       <c r="G13" s="11">
         <v>34</v>
       </c>
-      <c r="H13" s="22" t="s">
-        <v>128</v>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I13" s="16">
         <f>IF(F13="Clay",Input!$C$32*G13,0)</f>
@@ -13823,8 +13867,10 @@
       <c r="G14" s="11">
         <v>13</v>
       </c>
-      <c r="H14" s="22" t="s">
-        <v>129</v>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L</t>
+        </is>
       </c>
       <c r="I14" s="20">
         <f>IF(F14="Clay",Input!$C$32*G14,0)</f>
@@ -13874,8 +13920,10 @@
       <c r="G15" s="11">
         <v>17</v>
       </c>
-      <c r="H15" s="22" t="s">
-        <v>129</v>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L</t>
+        </is>
       </c>
       <c r="I15" s="16">
         <f>IF(F15="Clay",Input!$C$32*G15,0)</f>
@@ -13925,8 +13973,10 @@
       <c r="G16" s="11">
         <v>18</v>
       </c>
-      <c r="H16" s="22" t="s">
-        <v>129</v>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L</t>
+        </is>
       </c>
       <c r="I16" s="20">
         <f>IF(F16="Clay",Input!$C$32*G16,0)</f>
@@ -13976,8 +14026,10 @@
       <c r="G17" s="11">
         <v>19</v>
       </c>
-      <c r="H17" s="22" t="s">
-        <v>129</v>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L</t>
+        </is>
       </c>
       <c r="I17" s="16">
         <f>IF(F17="Clay",Input!$C$32*G17,0)</f>
@@ -14027,8 +14079,10 @@
       <c r="G18" s="11">
         <v>12</v>
       </c>
-      <c r="H18" s="22" t="s">
-        <v>129</v>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L</t>
+        </is>
       </c>
       <c r="I18" s="20">
         <f>IF(F18="Clay",Input!$C$32*G18,0)</f>
@@ -14078,8 +14132,10 @@
       <c r="G19" s="11">
         <v>42</v>
       </c>
-      <c r="H19" s="22" t="s">
-        <v>128</v>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I19" s="16">
         <f>IF(F19="Clay",Input!$C$32*G19,0)</f>
@@ -14129,8 +14185,10 @@
       <c r="G20" s="11">
         <v>49</v>
       </c>
-      <c r="H20" s="22" t="s">
-        <v>128</v>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I20" s="20">
         <f>IF(F20="Clay",Input!$C$32*G20,0)</f>
@@ -14180,8 +14238,10 @@
       <c r="G21" s="11">
         <v>49</v>
       </c>
-      <c r="H21" s="6" t="s">
-        <v>128</v>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I21" s="16">
         <f>IF(F21="Clay",Input!$C$32*G21,0)</f>
@@ -14231,8 +14291,10 @@
       <c r="G22" s="11">
         <v>44</v>
       </c>
-      <c r="H22" s="6" t="s">
-        <v>128</v>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I22" s="20">
         <f>IF(F22="Clay",Input!$C$32*G22,0)</f>
@@ -14280,8 +14342,10 @@
       <c r="G23" s="11">
         <v>20</v>
       </c>
-      <c r="H23" s="6" t="s">
-        <v>128</v>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I23" s="16">
         <f>IF(F23="Clay",Input!$C$32*G23,0)</f>
@@ -14329,8 +14393,10 @@
       <c r="G24" s="11">
         <v>21</v>
       </c>
-      <c r="H24" s="6" t="s">
-        <v>128</v>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I24" s="20">
         <f>IF(F24="Clay",Input!$C$32*G24,0)</f>
@@ -14378,8 +14444,10 @@
       <c r="G25" s="11">
         <v>21</v>
       </c>
-      <c r="H25" s="6" t="s">
-        <v>128</v>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I25" s="16">
         <f>IF(F25="Clay",Input!$C$32*G25,0)</f>
@@ -14427,8 +14495,10 @@
       <c r="G26" s="11">
         <v>48</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>128</v>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I26" s="20">
         <f>IF(F26="Clay",Input!$C$32*G26,0)</f>
@@ -14476,8 +14546,10 @@
       <c r="G27" s="11">
         <v>50</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>128</v>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I27" s="16">
         <f>IF(F27="Clay",Input!$C$32*G27,0)</f>
@@ -14525,8 +14597,10 @@
       <c r="G28" s="11">
         <v>50</v>
       </c>
-      <c r="H28" s="6" t="s">
-        <v>128</v>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I28" s="20">
         <f>IF(F28="Clay",Input!$C$32*G28,0)</f>
@@ -14574,8 +14648,10 @@
       <c r="G29" s="11">
         <v>50</v>
       </c>
-      <c r="H29" s="6" t="s">
-        <v>128</v>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I29" s="16">
         <f>IF(F29="Clay",Input!$C$32*G29,0)</f>
@@ -14623,8 +14699,10 @@
       <c r="G30" s="11">
         <v>50</v>
       </c>
-      <c r="H30" s="6" t="s">
-        <v>128</v>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I30" s="20">
         <f>IF(F30="Clay",Input!$C$32*G30,0)</f>
@@ -14672,8 +14750,10 @@
       <c r="G31" s="11">
         <v>50</v>
       </c>
-      <c r="H31" s="6" t="s">
-        <v>128</v>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I31" s="16">
         <f>IF(F31="Clay",Input!$C$32*G31,0)</f>
@@ -14721,8 +14801,10 @@
       <c r="G32" s="11">
         <v>50</v>
       </c>
-      <c r="H32" s="6" t="s">
-        <v>128</v>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I32" s="20">
         <f>IF(F32="Clay",Input!$C$32*G32,0)</f>
@@ -14770,8 +14852,10 @@
       <c r="G33" s="11">
         <v>50</v>
       </c>
-      <c r="H33" s="6" t="s">
-        <v>128</v>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I33" s="16">
         <f>IF(F33="Clay",Input!$C$32*G33,0)</f>
@@ -14819,8 +14903,10 @@
       <c r="G34" s="11">
         <v>50</v>
       </c>
-      <c r="H34" s="6" t="s">
-        <v>128</v>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I34" s="20">
         <f>IF(F34="Clay",Input!$C$32*G34,0)</f>
@@ -14868,8 +14954,10 @@
       <c r="G35" s="11">
         <v>50</v>
       </c>
-      <c r="H35" s="6" t="s">
-        <v>128</v>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I35" s="16">
         <f>IF(F35="Clay",Input!$C$32*G35,0)</f>
@@ -14917,8 +15005,10 @@
       <c r="G36" s="11">
         <v>50</v>
       </c>
-      <c r="H36" s="6" t="s">
-        <v>128</v>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I36" s="20">
         <f>IF(F36="Clay",Input!$C$32*G36,0)</f>
@@ -14966,8 +15056,10 @@
       <c r="G37" s="11">
         <v>33</v>
       </c>
-      <c r="H37" s="6" t="s">
-        <v>128</v>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I37" s="16">
         <f>IF(F37="Clay",Input!$C$32*G37,0)</f>
@@ -15015,8 +15107,10 @@
       <c r="G38" s="11">
         <v>36</v>
       </c>
-      <c r="H38" s="6" t="s">
-        <v>128</v>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I38" s="20">
         <f>IF(F38="Clay",Input!$C$32*G38,0)</f>
@@ -15064,8 +15158,10 @@
       <c r="G39" s="11">
         <v>31</v>
       </c>
-      <c r="H39" s="6" t="s">
-        <v>128</v>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I39" s="16">
         <f>IF(F39="Clay",Input!$C$32*G39,0)</f>
@@ -15113,8 +15209,10 @@
       <c r="G40" s="11">
         <v>30</v>
       </c>
-      <c r="H40" s="6" t="s">
-        <v>128</v>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I40" s="20">
         <f>IF(F40="Clay",Input!$C$32*G40,0)</f>
@@ -15162,8 +15260,10 @@
       <c r="G41" s="11">
         <v>34</v>
       </c>
-      <c r="H41" s="6" t="s">
-        <v>128</v>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I41" s="16">
         <f>IF(F41="Clay",Input!$C$32*G41,0)</f>
@@ -15211,8 +15311,10 @@
       <c r="G42" s="11">
         <v>31</v>
       </c>
-      <c r="H42" s="6" t="s">
-        <v>128</v>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I42" s="20">
         <f>IF(F42="Clay",Input!$C$32*G42,0)</f>
@@ -15260,8 +15362,10 @@
       <c r="G43" s="11">
         <v>29</v>
       </c>
-      <c r="H43" s="6" t="s">
-        <v>128</v>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I43" s="16">
         <f>IF(F43="Clay",Input!$C$32*G43,0)</f>
@@ -15309,8 +15413,10 @@
       <c r="G44" s="11">
         <v>25</v>
       </c>
-      <c r="H44" s="6" t="s">
-        <v>128</v>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I44" s="20">
         <f>IF(F44="Clay",Input!$C$32*G44,0)</f>
@@ -15358,8 +15464,10 @@
       <c r="G45" s="11">
         <v>35</v>
       </c>
-      <c r="H45" s="6" t="s">
-        <v>128</v>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I45" s="16">
         <f>IF(F45="Clay",Input!$C$32*G45,0)</f>
@@ -15407,8 +15515,10 @@
       <c r="G46" s="11">
         <v>42</v>
       </c>
-      <c r="H46" s="6" t="s">
-        <v>128</v>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I46" s="20">
         <f>IF(F46="Clay",Input!$C$32*G46,0)</f>
@@ -15456,8 +15566,10 @@
       <c r="G47" s="11">
         <v>46</v>
       </c>
-      <c r="H47" s="6" t="s">
-        <v>128</v>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NL</t>
+        </is>
       </c>
       <c r="I47" s="16">
         <f>IF(F47="Clay",Input!$C$32*G47,0)</f>

</xml_diff>

<commit_message>
PBCP rev4: uniform trial loads 3000/600/500 kN for all boreholes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVMNJXhKJM4HyR9gsSXKh
</commit_message>
<xml_diff>
--- a/deliverables/PBCP-BH-01_rev4.xlsx
+++ b/deliverables/PBCP-BH-01_rev4.xlsx
@@ -13232,14 +13232,14 @@
         <v>9</v>
       </c>
       <c r="C48" s="14">
-        <v>5152.9</v>
+        <v>3000.0</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, ASD2(max) - beban lama, update dgn GROUP beban revisi</t>
+          <t xml:space="preserve">beban seragam semua BH (sama dengan BH-03) - update dgn GROUP beban revisi</t>
         </is>
       </c>
     </row>
@@ -13251,14 +13251,14 @@
         <v>13</v>
       </c>
       <c r="C49" s="14">
-        <v>1583.9</v>
+        <v>600.0</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, LRFD3 - beban lama, update dgn GROUP beban revisi</t>
+          <t xml:space="preserve">beban seragam semua BH (sama dengan BH-03) - update dgn GROUP beban revisi</t>
         </is>
       </c>
     </row>
@@ -13270,14 +13270,14 @@
         <v>18</v>
       </c>
       <c r="C50" s="14">
-        <v>1101.5</v>
+        <v>500.0</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GROUP WPD 2 cellar 4x1, ASD1 (DL) - beban lama, update dgn GROUP beban revisi</t>
+          <t xml:space="preserve">beban seragam semua BH (sama dengan BH-03) - update dgn GROUP beban revisi</t>
         </is>
       </c>
     </row>
@@ -13296,7 +13296,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GROUP: tidak ada tiang tarik pada kombinasi yang ditinjau</t>
+          <t xml:space="preserve">tidak ada tiang tarik pada kombinasi yang ditinjau</t>
         </is>
       </c>
     </row>

</xml_diff>